<commit_message>
Fine tuning of plot layouts and models
Title says it all
</commit_message>
<xml_diff>
--- a/Data Analysis/1_Data/MainDomDiff.xlsx
+++ b/Data Analysis/1_Data/MainDomDiff.xlsx
@@ -2032,7 +2032,7 @@
         <v>453.828929076185</v>
       </c>
       <c r="D80">
-        <v>893.2258059999973</v>
+        <v>848.8764879999983</v>
       </c>
       <c r="E80" t="inlineStr">
         <is>
@@ -2143,7 +2143,7 @@
         <v>600.2987023647282</v>
       </c>
       <c r="D86">
-        <v>1079.088475000001</v>
+        <v>1096.1901727</v>
       </c>
       <c r="E86" t="inlineStr">
         <is>
@@ -2164,7 +2164,7 @@
         <v>337.121001145318</v>
       </c>
       <c r="D87">
-        <v>428.0145519999981</v>
+        <v>447.2937850000007</v>
       </c>
       <c r="E87" t="inlineStr">
         <is>
@@ -2203,7 +2203,7 @@
         <v>237.413509731037</v>
       </c>
       <c r="D89">
-        <v>-160.8030150000016</v>
+        <v>-194.9398349999993</v>
       </c>
       <c r="E89" t="inlineStr">
         <is>
@@ -2278,7 +2278,7 @@
         <v>65.15355448309538</v>
       </c>
       <c r="D93">
-        <v>-89.64040127499999</v>
+        <v>-194.6454993249984</v>
       </c>
       <c r="E93" t="inlineStr">
         <is>
@@ -2299,7 +2299,7 @@
         <v>318.0034539887487</v>
       </c>
       <c r="D94">
-        <v>721.4567737250006</v>
+        <v>600.3867187249998</v>
       </c>
       <c r="E94" t="inlineStr">
         <is>
@@ -2338,7 +2338,7 @@
         <v>243.8104367429125</v>
       </c>
       <c r="D96">
-        <v>107.2126987249998</v>
+        <v>-1.691360725000656</v>
       </c>
       <c r="E96" t="inlineStr">
         <is>
@@ -2359,7 +2359,7 @@
         <v>236.5240589428544</v>
       </c>
       <c r="D97">
-        <v>245.4405729499985</v>
+        <v>141.5645757499995</v>
       </c>
       <c r="E97" t="inlineStr">
         <is>
@@ -2380,7 +2380,7 @@
         <v>265.6750654253195</v>
       </c>
       <c r="D98">
-        <v>864.8655609499993</v>
+        <v>749.8983729500003</v>
       </c>
       <c r="E98" t="inlineStr">
         <is>
@@ -2401,7 +2401,7 @@
         <v>618.6941042076976</v>
       </c>
       <c r="D99">
-        <v>1328.438662999998</v>
+        <v>1251.405361999999</v>
       </c>
       <c r="E99" t="inlineStr">
         <is>
@@ -2458,7 +2458,7 @@
         <v>253.8833194137616</v>
       </c>
       <c r="D102">
-        <v>-372.0475095000011</v>
+        <v>-281.6896307999986</v>
       </c>
       <c r="E102" t="inlineStr">
         <is>
@@ -2479,7 +2479,7 @@
         <v>508.2722460836613</v>
       </c>
       <c r="D103">
-        <v>-460.7442240000004</v>
+        <v>-371.824670399999</v>
       </c>
       <c r="E103" t="inlineStr">
         <is>
@@ -2518,7 +2518,7 @@
         <v>601.0508871522345</v>
       </c>
       <c r="D105">
-        <v>1197.072097749999</v>
+        <v>1308.6591751</v>
       </c>
       <c r="E105" t="inlineStr">
         <is>
@@ -2539,7 +2539,7 @@
         <v>179.6038126892239</v>
       </c>
       <c r="D106">
-        <v>-5.830776500000502</v>
+        <v>-100.5679001000011</v>
       </c>
       <c r="E106" t="inlineStr">
         <is>
@@ -2560,7 +2560,7 @@
         <v>359.5747366146593</v>
       </c>
       <c r="D107">
-        <v>644.6568144999978</v>
+        <v>538.6719435999995</v>
       </c>
       <c r="E107" t="inlineStr">
         <is>
@@ -2581,7 +2581,7 @@
         <v>444.3538559888651</v>
       </c>
       <c r="D108">
-        <v>1017.0797485</v>
+        <v>904.6552174000002</v>
       </c>
       <c r="E108" t="inlineStr">
         <is>
@@ -2602,7 +2602,7 @@
         <v>337.4592058675807</v>
       </c>
       <c r="D109">
-        <v>1375.02160275</v>
+        <v>1421.384213550001</v>
       </c>
       <c r="E109" t="inlineStr">
         <is>
@@ -2659,7 +2659,7 @@
         <v>235.2127087553794</v>
       </c>
       <c r="D112">
-        <v>7.098722500000926</v>
+        <v>21.21688885000088</v>
       </c>
       <c r="E112" t="inlineStr">
         <is>
@@ -2698,7 +2698,7 @@
         <v>446.5076911021554</v>
       </c>
       <c r="D114">
-        <v>360.7547319999983</v>
+        <v>379.7759349999988</v>
       </c>
       <c r="E114" t="inlineStr">
         <is>
@@ -2737,7 +2737,7 @@
         <v>744.0588730597303</v>
       </c>
       <c r="D116">
-        <v>1191.360195</v>
+        <v>1148.66538</v>
       </c>
       <c r="E116" t="inlineStr">
         <is>
@@ -2776,7 +2776,7 @@
         <v>543.522889947967</v>
       </c>
       <c r="D118">
-        <v>1607.432655</v>
+        <v>1562.104470000002</v>
       </c>
       <c r="E118" t="inlineStr">
         <is>
@@ -2797,7 +2797,7 @@
         <v>306.9640902724445</v>
       </c>
       <c r="D119">
-        <v>-592.344465</v>
+        <v>-623.7500099999995</v>
       </c>
       <c r="E119" t="inlineStr">
         <is>
@@ -2890,7 +2890,7 @@
         <v>418.734195783599</v>
       </c>
       <c r="D124">
-        <v>1143.114562999998</v>
+        <v>1068.032042</v>
       </c>
       <c r="E124" t="inlineStr">
         <is>
@@ -2929,7 +2929,7 @@
         <v>247.4962054893521</v>
       </c>
       <c r="D126">
-        <v>1447.046086999999</v>
+        <v>1368.7642868</v>
       </c>
       <c r="E126" t="inlineStr">
         <is>
@@ -2968,7 +2968,7 @@
         <v>212.981337090379</v>
       </c>
       <c r="D128">
-        <v>535.7404604999998</v>
+        <v>640.8192251999998</v>
       </c>
       <c r="E128" t="inlineStr">
         <is>
@@ -2989,7 +2989,7 @@
         <v>457.0187511172023</v>
       </c>
       <c r="D129">
-        <v>703.4175044999992</v>
+        <v>811.2153564000007</v>
       </c>
       <c r="E129" t="inlineStr">
         <is>
@@ -3028,7 +3028,7 @@
         <v>269.3058999739118</v>
       </c>
       <c r="D131">
-        <v>82.92123449999877</v>
+        <v>-30.85797240000005</v>
       </c>
       <c r="E131" t="inlineStr">
         <is>
@@ -3049,7 +3049,7 @@
         <v>552.9978477879682</v>
       </c>
       <c r="D132">
-        <v>1263.675298500001</v>
+        <v>1124.64297</v>
       </c>
       <c r="E132" t="inlineStr">
         <is>
@@ -3070,7 +3070,7 @@
         <v>202.7281830201069</v>
       </c>
       <c r="D133">
-        <v>19.23915599999988</v>
+        <v>-93.17806424999823</v>
       </c>
       <c r="E133" t="inlineStr">
         <is>
@@ -3163,7 +3163,7 @@
         <v>245.4562153672685</v>
       </c>
       <c r="D138">
-        <v>486.8967082500012</v>
+        <v>779.0276968500004</v>
       </c>
       <c r="E138" t="inlineStr">
         <is>
@@ -3238,7 +3238,7 @@
         <v>304.439527026046</v>
       </c>
       <c r="D142">
-        <v>-993.7067856750024</v>
+        <v>-851.933382525002</v>
       </c>
       <c r="E142" t="inlineStr">
         <is>
@@ -3295,7 +3295,7 @@
         <v>568.9771421242084</v>
       </c>
       <c r="D145">
-        <v>413.195425499999</v>
+        <v>746.4886406999993</v>
       </c>
       <c r="E145" t="inlineStr">
         <is>
@@ -3316,7 +3316,7 @@
         <v>250.3710904358568</v>
       </c>
       <c r="D146">
-        <v>811.0674832500013</v>
+        <v>920.7122443500004</v>
       </c>
       <c r="E146" t="inlineStr">
         <is>
@@ -3373,7 +3373,7 @@
         <v>141.0811979857205</v>
       </c>
       <c r="D149">
-        <v>-343.8933560000034</v>
+        <v>-98.86338320000117</v>
       </c>
       <c r="E149" t="inlineStr">
         <is>
@@ -3394,7 +3394,7 @@
         <v>570.3699114310849</v>
       </c>
       <c r="D150">
-        <v>1749.455874500002</v>
+        <v>1545.549039500002</v>
       </c>
       <c r="E150" t="inlineStr">
         <is>
@@ -3451,7 +3451,7 @@
         <v>69.68062171620353</v>
       </c>
       <c r="D153">
-        <v>-544.5011280000006</v>
+        <v>-546.7792035000001</v>
       </c>
       <c r="E153" t="inlineStr">
         <is>
@@ -3526,7 +3526,7 @@
         <v>338.0676326165602</v>
       </c>
       <c r="D157">
-        <v>-1199.719635000002</v>
+        <v>-1199.031372000001</v>
       </c>
       <c r="E157" t="inlineStr">
         <is>
@@ -3565,7 +3565,7 @@
         <v>437.5855439183227</v>
       </c>
       <c r="D159">
-        <v>1187.625164999997</v>
+        <v>1188.650147999999</v>
       </c>
       <c r="E159" t="inlineStr">
         <is>
@@ -3604,7 +3604,7 @@
         <v>267.4119599578207</v>
       </c>
       <c r="D161">
-        <v>-191.4811350000004</v>
+        <v>-18.36298859999903</v>
       </c>
       <c r="E161" t="inlineStr">
         <is>
@@ -3643,7 +3643,7 @@
         <v>619.2352319959074</v>
       </c>
       <c r="D163">
-        <v>607.7201250000013</v>
+        <v>806.3512347000011</v>
       </c>
       <c r="E163" t="inlineStr">
         <is>
@@ -3664,7 +3664,7 @@
         <v>611.1551248746335</v>
       </c>
       <c r="D164">
-        <v>97.13914500000149</v>
+        <v>279.4709388000008</v>
       </c>
       <c r="E164" t="inlineStr">
         <is>
@@ -3721,7 +3721,7 @@
         <v>272.4008841800821</v>
       </c>
       <c r="D167">
-        <v>-248.9339392499998</v>
+        <v>7.34028554999968</v>
       </c>
       <c r="E167" t="inlineStr">
         <is>
@@ -3778,7 +3778,7 @@
         <v>442.2871984140043</v>
       </c>
       <c r="D170">
-        <v>483.8643524999992</v>
+        <v>820.650726600002</v>
       </c>
       <c r="E170" t="inlineStr">
         <is>
@@ -3853,7 +3853,7 @@
         <v>224.7123309110494</v>
       </c>
       <c r="D174">
-        <v>331.4731612500017</v>
+        <v>432.6917605500009</v>
       </c>
       <c r="E174" t="inlineStr">
         <is>
@@ -3910,7 +3910,7 @@
         <v>530.3218208169246</v>
       </c>
       <c r="D177">
-        <v>1256.491968999996</v>
+        <v>1572.698400999998</v>
       </c>
       <c r="E177" t="inlineStr">
         <is>
@@ -3949,7 +3949,7 @@
         <v>410.3996813284041</v>
       </c>
       <c r="D179">
-        <v>834.3596164999996</v>
+        <v>654.3563513000011</v>
       </c>
       <c r="E179" t="inlineStr">
         <is>
@@ -3988,7 +3988,7 @@
         <v>436.2224779515712</v>
       </c>
       <c r="D181">
-        <v>852.9033420000002</v>
+        <v>850.057600499999</v>
       </c>
       <c r="E181" t="inlineStr">
         <is>
@@ -4009,7 +4009,7 @@
         <v>535.3352371018603</v>
       </c>
       <c r="D182">
-        <v>1615.799689499999</v>
+        <v>1612.6440375</v>
       </c>
       <c r="E182" t="inlineStr">
         <is>
@@ -4030,7 +4030,7 @@
         <v>251.8449287383603</v>
       </c>
       <c r="D183">
-        <v>-300.906534000001</v>
+        <v>213.6283439999989</v>
       </c>
       <c r="E183" t="inlineStr">
         <is>
@@ -4051,7 +4051,7 @@
         <v>297.7463178859696</v>
       </c>
       <c r="D184">
-        <v>728.5914419999987</v>
+        <v>1337.323300799999</v>
       </c>
       <c r="E184" t="inlineStr">
         <is>
@@ -4072,7 +4072,7 @@
         <v>429.7470407540609</v>
       </c>
       <c r="D185">
-        <v>650.3485109999999</v>
+        <v>1251.921299999999</v>
       </c>
       <c r="E185" t="inlineStr">
         <is>
@@ -4129,7 +4129,7 @@
         <v>180.0178036519824</v>
       </c>
       <c r="D188">
-        <v>99.38448180000026</v>
+        <v>708.2651562000004</v>
       </c>
       <c r="E188" t="inlineStr">
         <is>
@@ -4150,7 +4150,7 @@
         <v>327.0545203412071</v>
       </c>
       <c r="D189">
-        <v>1273.0688898</v>
+        <v>2015.272530600002</v>
       </c>
       <c r="E189" t="inlineStr">
         <is>
@@ -4189,7 +4189,7 @@
         <v>495.354024359066</v>
       </c>
       <c r="D191">
-        <v>1771.981271299996</v>
+        <v>1782.373585099998</v>
       </c>
       <c r="E191" t="inlineStr">
         <is>
@@ -4264,7 +4264,7 @@
         <v>206.2718142247142</v>
       </c>
       <c r="D195">
-        <v>-333.5248200000002</v>
+        <v>219.0162665999989</v>
       </c>
       <c r="E195" t="inlineStr">
         <is>
@@ -4285,7 +4285,7 @@
         <v>477.0983926930683</v>
       </c>
       <c r="D196">
-        <v>828.6686520000007</v>
+        <v>1486.9453818</v>
       </c>
       <c r="E196" t="inlineStr">
         <is>
@@ -4324,7 +4324,7 @@
         <v>259.720514230434</v>
       </c>
       <c r="D198">
-        <v>219.7694579999981</v>
+        <v>783.5731697999988</v>
       </c>
       <c r="E198" t="inlineStr">
         <is>
@@ -4345,7 +4345,7 @@
         <v>449.0570625434337</v>
       </c>
       <c r="D199">
-        <v>801.0824999999992</v>
+        <v>1416.143377199998</v>
       </c>
       <c r="E199" t="inlineStr">
         <is>
@@ -4366,7 +4366,7 @@
         <v>513.7793269978939</v>
       </c>
       <c r="D200">
-        <v>1052.230236</v>
+        <v>1689.436016399997</v>
       </c>
       <c r="E200" t="inlineStr">
         <is>
@@ -4531,7 +4531,7 @@
         <v>460.2469717114527</v>
       </c>
       <c r="D209">
-        <v>1799.2554083</v>
+        <v>1809.685365199999</v>
       </c>
       <c r="E209" t="inlineStr">
         <is>
@@ -4552,7 +4552,7 @@
         <v>283.5717566306607</v>
       </c>
       <c r="D210">
-        <v>1310.946260299998</v>
+        <v>1320.702264799997</v>
       </c>
       <c r="E210" t="inlineStr">
         <is>
@@ -4573,7 +4573,7 @@
         <v>413.2996415144439</v>
       </c>
       <c r="D211">
-        <v>-304.9812120000007</v>
+        <v>250.1567544</v>
       </c>
       <c r="E211" t="inlineStr">
         <is>
@@ -4612,7 +4612,7 @@
         <v>473.6020889042558</v>
       </c>
       <c r="D213">
-        <v>1296.971141999999</v>
+        <v>1955.756904599998</v>
       </c>
       <c r="E213" t="inlineStr">
         <is>
@@ -4633,7 +4633,7 @@
         <v>157.0890676499875</v>
       </c>
       <c r="D214">
-        <v>-99.0533249999998</v>
+        <v>-160.8970769999985</v>
       </c>
       <c r="E214" t="inlineStr">
         <is>
@@ -4690,7 +4690,7 @@
         <v>280.3394055703297</v>
       </c>
       <c r="D217">
-        <v>-20.07272100000215</v>
+        <v>520.1578823999977</v>
       </c>
       <c r="E217" t="inlineStr">
         <is>
@@ -4873,7 +4873,7 @@
         <v>453.6761392600661</v>
       </c>
       <c r="D227">
-        <v>1627.297079299998</v>
+        <v>1637.489703499997</v>
       </c>
       <c r="E227" t="inlineStr">
         <is>
@@ -4894,7 +4894,7 @@
         <v>558.1751881825418</v>
       </c>
       <c r="D228">
-        <v>965.9903879999988</v>
+        <v>1636.760564399999</v>
       </c>
       <c r="E228" t="inlineStr">
         <is>
@@ -4951,7 +4951,7 @@
         <v>394.0227101168635</v>
       </c>
       <c r="D231">
-        <v>1531.745868</v>
+        <v>2211.232846799998</v>
       </c>
       <c r="E231" t="inlineStr">
         <is>
@@ -5008,7 +5008,7 @@
         <v>317.5762589370038</v>
       </c>
       <c r="D234">
-        <v>2088.206411999999</v>
+        <v>1562.0473557</v>
       </c>
       <c r="E234" t="inlineStr">
         <is>
@@ -5029,7 +5029,7 @@
         <v>261.2922998809232</v>
       </c>
       <c r="D235">
-        <v>1411.221701999999</v>
+        <v>939.7552152</v>
       </c>
       <c r="E235" t="inlineStr">
         <is>
@@ -5104,7 +5104,7 @@
         <v>503.874324646469</v>
       </c>
       <c r="D239">
-        <v>1990.989217499999</v>
+        <v>2302.872896699998</v>
       </c>
       <c r="E239" t="inlineStr">
         <is>
@@ -5143,7 +5143,7 @@
         <v>165.7618580880668</v>
       </c>
       <c r="D241">
-        <v>287.4671055000004</v>
+        <v>341.0062992000011</v>
       </c>
       <c r="E241" t="inlineStr">
         <is>
@@ -5182,7 +5182,7 @@
         <v>223.8066832854715</v>
       </c>
       <c r="D243">
-        <v>2088.645062999999</v>
+        <v>1562.45056875</v>
       </c>
       <c r="E243" t="inlineStr">
         <is>
@@ -5203,7 +5203,7 @@
         <v>252.7978394291253</v>
       </c>
       <c r="D244">
-        <v>1086.473745</v>
+        <v>641.2431538499989</v>
       </c>
       <c r="E244" t="inlineStr">
         <is>
@@ -5224,7 +5224,7 @@
         <v>473.3503413854864</v>
       </c>
       <c r="D245">
-        <v>2031.620433</v>
+        <v>1510.032872249998</v>
       </c>
       <c r="E245" t="inlineStr">
         <is>
@@ -5281,7 +5281,7 @@
         <v>341.9850607213597</v>
       </c>
       <c r="D248">
-        <v>1212.237933000001</v>
+        <v>1489.201616249998</v>
       </c>
       <c r="E248" t="inlineStr">
         <is>
@@ -5302,7 +5302,7 @@
         <v>195.8540186201228</v>
       </c>
       <c r="D249">
-        <v>734.9478554999989</v>
+        <v>990.509368499998</v>
       </c>
       <c r="E249" t="inlineStr">
         <is>
@@ -5359,7 +5359,7 @@
         <v>585.6839740724151</v>
       </c>
       <c r="D252">
-        <v>2654.747145</v>
+        <v>2733.697819350003</v>
       </c>
       <c r="E252" t="inlineStr">
         <is>
@@ -5416,7 +5416,7 @@
         <v>311.4068972761521</v>
       </c>
       <c r="D255">
-        <v>1567.606365</v>
+        <v>1446.081326250001</v>
       </c>
       <c r="E255" t="inlineStr">
         <is>
@@ -5437,7 +5437,7 @@
         <v>561.1679782522129</v>
       </c>
       <c r="D256">
-        <v>1824.5080785</v>
+        <v>1995.616802550001</v>
       </c>
       <c r="E256" t="inlineStr">
         <is>
@@ -5512,7 +5512,7 @@
         <v>438.2481548528709</v>
       </c>
       <c r="D260">
-        <v>1129.4863395</v>
+        <v>1571.210138249999</v>
       </c>
       <c r="E260" t="inlineStr">
         <is>
@@ -5551,7 +5551,7 @@
         <v>179.8286902181561</v>
       </c>
       <c r="D262">
-        <v>483.7527835000016</v>
+        <v>693.3132113500003</v>
       </c>
       <c r="E262" t="inlineStr">
         <is>
@@ -5572,7 +5572,7 @@
         <v>194.4406132451904</v>
       </c>
       <c r="D263">
-        <v>1318.950906</v>
+        <v>1202.667874800002</v>
       </c>
       <c r="E263" t="inlineStr">
         <is>
@@ -5611,7 +5611,7 @@
         <v>574.0342781949324</v>
       </c>
       <c r="D265">
-        <v>2766.002178</v>
+        <v>2619.213266400002</v>
       </c>
       <c r="E265" t="inlineStr">
         <is>
@@ -5650,7 +5650,7 @@
         <v>278.8805656457188</v>
       </c>
       <c r="D267">
-        <v>568.3274534999995</v>
+        <v>705.5697400500009</v>
       </c>
       <c r="E267" t="inlineStr">
         <is>
@@ -5761,7 +5761,7 @@
         <v>156.4544841570865</v>
       </c>
       <c r="D273">
-        <v>536.4183535000018</v>
+        <v>748.1880854500001</v>
       </c>
       <c r="E273" t="inlineStr">
         <is>
@@ -5818,7 +5818,7 @@
         <v>686.1627598290961</v>
       </c>
       <c r="D276">
-        <v>1928.127863500001</v>
+        <v>2198.279371750002</v>
       </c>
       <c r="E276" t="inlineStr">
         <is>
@@ -5839,7 +5839,7 @@
         <v>329.2885417839064</v>
       </c>
       <c r="D277">
-        <v>1461.028263000001</v>
+        <v>1791.712007999999</v>
       </c>
       <c r="E277" t="inlineStr">
         <is>
@@ -5878,7 +5878,7 @@
         <v>413.1976218228556</v>
       </c>
       <c r="D279">
-        <v>1496.434919999999</v>
+        <v>1829.000819999999</v>
       </c>
       <c r="E279" t="inlineStr">
         <is>
@@ -5917,7 +5917,7 @@
         <v>209.1876306057004</v>
       </c>
       <c r="D281">
-        <v>378.0527460000002</v>
+        <v>651.1674359999995</v>
       </c>
       <c r="E281" t="inlineStr">
         <is>
@@ -5956,7 +5956,7 @@
         <v>408.9694871658746</v>
       </c>
       <c r="D283">
-        <v>1509.163759500002</v>
+        <v>1842.406301999999</v>
       </c>
       <c r="E283" t="inlineStr">
         <is>
@@ -5995,7 +5995,7 @@
         <v>313.3708268261595</v>
       </c>
       <c r="D285">
-        <v>1685.611810499999</v>
+        <v>2028.234017999999</v>
       </c>
       <c r="E285" t="inlineStr">
         <is>

</xml_diff>